<commit_message>
- Fix values for Q47 (2021): swapped "bank" and "criminals" responses. - Fix labels for created income variables (resp_household_income and resp_mean_household_income): added "remedy order of magnitude errors". - Fix household size label: added "winsorized at 99%". — Add link in further reading.
</commit_message>
<xml_diff>
--- a/data/supplementary_data/english_version/all_waves_variables.xlsx
+++ b/data/supplementary_data/english_version/all_waves_variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kuchakov/R/_criminology/create_victimization_data/data/supplementary_data/english_version/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kuchakov/R/_criminology/create_victimization_data/_repo/data/supplementary_data/english_version/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F44C851-37ED-7143-AE9B-526F9D24A9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268A09D2-670E-4D45-BA61-404077C8C3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8300" yWindow="2540" windowWidth="23080" windowHeight="15100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="312">
   <si>
     <t>type</t>
   </si>
@@ -928,9 +928,6 @@
     <t>Thank you. May we call you again in three years regarding the same topic?</t>
   </si>
   <si>
-    <t>Total monthly household income (winsorized at 99%)</t>
-  </si>
-  <si>
     <t>weight</t>
   </si>
   <si>
@@ -952,7 +949,13 @@
     <t>resp_mean_household_income</t>
   </si>
   <si>
-    <t>Average income of the respondent’s household member</t>
+    <t>Total monthly household income (remedy order of magnitude errors and winsorized at 99%)</t>
+  </si>
+  <si>
+    <t>Average income of the respondent’s household member (remedy order of magnitude errors and winsorized at 99%)</t>
+  </si>
+  <si>
+    <t>Household size (winsorized at 99%)</t>
   </si>
 </sst>
 </file>
@@ -1989,29 +1992,29 @@
         <v>4</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -2396,7 +2399,7 @@
         <v>4</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>226</v>
+        <v>311</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -2407,12 +2410,12 @@
         <v>4</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
@@ -2995,7 +2998,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B155" t="s">
         <v>4</v>

</xml_diff>